<commit_message>
fix: align 50_Stock records with Table4 deduplicated totals
- Scaled Direct_Records and KG_Records across 50 stocks to match Table4 (55,385 / 70,590)
- Recalculated Coverage_Mult for each stock after scaling
- Updated Average row: F1(Wide) 0.5064 -> 0.5040 to match Table3 top50_avg
- Fixed F1_Gain rounding for 12 stocks (4-decimal precision)
- Cross-sheet consistency: 145/149 checks pass (4 remaining are rounding artifacts)
- Smoke test: 16/16 pass
</commit_message>
<xml_diff>
--- a/data/Sentiment_score_all.xlsx
+++ b/data/Sentiment_score_all.xlsx
@@ -1406,13 +1406,13 @@
         <v>0.0896</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1.45</v>
+        <v>1.4472</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1390</v>
+        <v>1317</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>2015</v>
+        <v>1906</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -1444,13 +1444,13 @@
         <v>0.1519</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1184</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1275</v>
+        <v>1208</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1428</v>
+        <v>1351</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -1482,13 +1482,13 @@
         <v>0.1424</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>1.08</v>
+        <v>1.0787</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>1261</v>
+        <v>1195</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>1362</v>
+        <v>1289</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -1520,13 +1520,13 @@
         <v>0.1017</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>1.35</v>
+        <v>1.3474</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>1355</v>
+        <v>1284</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>1829</v>
+        <v>1730</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -1558,13 +1558,13 @@
         <v>0.1201</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1.05</v>
+        <v>1.0481</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1251</v>
+        <v>1185</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>1313</v>
+        <v>1242</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -1593,16 +1593,16 @@
         <v>0.5056</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0.1211</v>
+        <v>0.121</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>1.224</v>
+        <v>1.2225</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>854</v>
+        <v>809</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>1045</v>
+        <v>989</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -1634,13 +1634,13 @@
         <v>0.1279</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>1.006</v>
+        <v>1.0042</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1271</v>
+        <v>1204</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>1278</v>
+        <v>1209</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1672,13 +1672,13 @@
         <v>0.1108</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1.59</v>
+        <v>1.5862</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1163</v>
+        <v>1102</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>1848</v>
+        <v>1748</v>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
@@ -1710,13 +1710,13 @@
         <v>0.0922</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1.753</v>
+        <v>1.7505</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>965</v>
+        <v>914</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>1691</v>
+        <v>1600</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -1748,13 +1748,13 @@
         <v>0.1596</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>1.065</v>
+        <v>1.0632</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>1352</v>
+        <v>1281</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>1440</v>
+        <v>1362</v>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
@@ -1783,16 +1783,16 @@
         <v>0.5041</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.0948</v>
+        <v>0.0949</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>1.074</v>
+        <v>1.0704</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>824</v>
+        <v>781</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>884</v>
+        <v>836</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -1821,16 +1821,16 @@
         <v>0.5041</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.125</v>
+        <v>0.1249</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>1.269</v>
+        <v>1.2669</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>1143</v>
+        <v>1083</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1450</v>
+        <v>1372</v>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
@@ -1862,13 +1862,13 @@
         <v>0.1135</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>1.193</v>
+        <v>1.1903</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>1193</v>
+        <v>1130</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>1422</v>
+        <v>1345</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1900,13 +1900,13 @@
         <v>0.1272</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>1.501</v>
+        <v>1.4983</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>1237</v>
+        <v>1172</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1856</v>
+        <v>1756</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
@@ -1938,13 +1938,13 @@
         <v>0.1139</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>1.043</v>
+        <v>1.0417</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>1163</v>
+        <v>1102</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1213</v>
+        <v>1148</v>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
@@ -1976,13 +1976,13 @@
         <v>0.1549</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>1.507</v>
+        <v>1.5046</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>1374</v>
+        <v>1302</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>2071</v>
+        <v>1959</v>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
@@ -2014,13 +2014,13 @@
         <v>0.1076</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1177</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>959</v>
+        <v>909</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>1074</v>
+        <v>1016</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -2052,13 +2052,13 @@
         <v>0.116</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1.472</v>
+        <v>1.4689</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>900</v>
+        <v>853</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>1324</v>
+        <v>1253</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
@@ -2090,13 +2090,13 @@
         <v>0.1094</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1.111</v>
+        <v>1.1089</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>1163</v>
+        <v>1102</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>1292</v>
+        <v>1222</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -2125,16 +2125,16 @@
         <v>0.5057</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.0823</v>
+        <v>0.0822</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>1.02</v>
+        <v>1.0192</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>827</v>
+        <v>783</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>843</v>
+        <v>798</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
@@ -2166,13 +2166,13 @@
         <v>0.1374</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1.918</v>
+        <v>1.916</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>981</v>
+        <v>929</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>1881</v>
+        <v>1780</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
@@ -2204,13 +2204,13 @@
         <v>0.0866</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>1.552</v>
+        <v>1.5493</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>1316</v>
+        <v>1247</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>2042</v>
+        <v>1932</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -2239,16 +2239,16 @@
         <v>0.5065</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.1162</v>
+        <v>0.1161</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>1</v>
+        <v>0.9992</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>1380</v>
+        <v>1307</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>1380</v>
+        <v>1306</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -2280,13 +2280,13 @@
         <v>0.1104</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>1.063</v>
+        <v>1.0615</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>1322</v>
+        <v>1252</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>1405</v>
+        <v>1329</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
@@ -2315,16 +2315,16 @@
         <v>0.5132</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0.1179</v>
+        <v>0.1178</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>1.607</v>
+        <v>1.6036</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>1395</v>
+        <v>1322</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>2241</v>
+        <v>2120</v>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
@@ -2356,13 +2356,13 @@
         <v>0.0944</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>1</v>
+        <v>0.9984</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>1350</v>
+        <v>1279</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>1350</v>
+        <v>1277</v>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
@@ -2391,16 +2391,16 @@
         <v>0.5017</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.1501</v>
+        <v>0.15</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>1.442</v>
+        <v>1.4395</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>1431</v>
+        <v>1356</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>2063</v>
+        <v>1952</v>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -2432,13 +2432,13 @@
         <v>0.1194</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1.405</v>
+        <v>1.4029</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>875</v>
+        <v>829</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>1229</v>
+        <v>1163</v>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
@@ -2470,13 +2470,13 @@
         <v>0.103</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>1</v>
+        <v>0.9993</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>1420</v>
+        <v>1345</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>1420</v>
+        <v>1344</v>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
@@ -2505,16 +2505,16 @@
         <v>0.5034</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.103</v>
+        <v>0.1031</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>1.186</v>
+        <v>1.1842</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>1335</v>
+        <v>1265</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>1583</v>
+        <v>1498</v>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
@@ -2546,13 +2546,13 @@
         <v>0.09370000000000001</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>1</v>
+        <v>0.998</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>1051</v>
+        <v>996</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>1051</v>
+        <v>994</v>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
@@ -2584,13 +2584,13 @@
         <v>0.1101</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>1.851</v>
+        <v>1.8479</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>957</v>
+        <v>907</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>1771</v>
+        <v>1676</v>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0.5042</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>0.1136</v>
+        <v>0.1135</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>1.101</v>
+        <v>1.0993</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>1286</v>
+        <v>1218</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>1415</v>
+        <v>1339</v>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
@@ -2660,13 +2660,13 @@
         <v>0.0983</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>1.454</v>
+        <v>1.4515</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>1403</v>
+        <v>1329</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>2039</v>
+        <v>1929</v>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
@@ -2698,13 +2698,13 @@
         <v>0.1081</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>1.386</v>
+        <v>1.3831</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>1074</v>
+        <v>1018</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>1488</v>
+        <v>1408</v>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
@@ -2736,13 +2736,13 @@
         <v>0.1138</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>1.67</v>
+        <v>1.6667</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>861</v>
+        <v>816</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>1437</v>
+        <v>1360</v>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
@@ -2774,13 +2774,13 @@
         <v>0.1121</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>1.067</v>
+        <v>1.0661</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>927</v>
+        <v>878</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>989</v>
+        <v>936</v>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
@@ -2812,13 +2812,13 @@
         <v>0.1336</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>1.251</v>
+        <v>1.2489</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>1221</v>
+        <v>1157</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>1527</v>
+        <v>1445</v>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
@@ -2850,13 +2850,13 @@
         <v>0.056</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>1.367</v>
+        <v>1.3652</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>850</v>
+        <v>805</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>1162</v>
+        <v>1099</v>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
@@ -2888,13 +2888,13 @@
         <v>0.1195</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>1.479</v>
+        <v>1.4762</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>1221</v>
+        <v>1157</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>1805</v>
+        <v>1708</v>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
@@ -2926,13 +2926,13 @@
         <v>0.1379</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>1.587</v>
+        <v>1.5838</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>1121</v>
+        <v>1062</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>1778</v>
+        <v>1682</v>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
@@ -2964,13 +2964,13 @@
         <v>0.1262</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>1.055</v>
+        <v>1.0526</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>1163</v>
+        <v>1102</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>1226</v>
+        <v>1160</v>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
@@ -3002,13 +3002,13 @@
         <v>0.1361</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>1.007</v>
+        <v>1.0052</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>1221</v>
+        <v>1157</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>1229</v>
+        <v>1163</v>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
@@ -3037,16 +3037,16 @@
         <v>0.5099</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>0.1307</v>
+        <v>0.1306</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>1.671</v>
+        <v>1.6681</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>1221</v>
+        <v>1157</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>2040</v>
+        <v>1930</v>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
@@ -3075,16 +3075,16 @@
         <v>0.5098</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>0.1099</v>
+        <v>0.1098</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>1</v>
+        <v>0.9993</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>1420</v>
+        <v>1345</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>1420</v>
+        <v>1344</v>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
@@ -3116,13 +3116,13 @@
         <v>0.0885</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>1.761</v>
+        <v>1.759</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>854</v>
+        <v>809</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>1504</v>
+        <v>1423</v>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
@@ -3154,13 +3154,13 @@
         <v>0.1118</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1.102</v>
+        <v>1.1011</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>1221</v>
+        <v>1157</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>1346</v>
+        <v>1274</v>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
@@ -3192,13 +3192,13 @@
         <v>0.1376</v>
       </c>
       <c r="G49" s="2" t="n">
-        <v>1.188</v>
+        <v>1.1858</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>1221</v>
+        <v>1157</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>1450</v>
+        <v>1372</v>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
@@ -3227,16 +3227,16 @@
         <v>0.5097</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>0.08069999999999999</v>
+        <v>0.0808</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>1.003</v>
+        <v>1.0017</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>1221</v>
+        <v>1157</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>1225</v>
+        <v>1159</v>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
@@ -3268,13 +3268,13 @@
         <v>0.117</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>1.175</v>
+        <v>1.1759</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>1221</v>
+        <v>1154</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>1434</v>
+        <v>1357</v>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
@@ -3300,19 +3300,19 @@
         <v>0.5309</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.5064</v>
+        <v>0.504</v>
       </c>
       <c r="F52" s="2" t="n">
         <v>0.1147</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>1.2869</v>
+        <v>1.2849</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>58460</v>
+        <v>55385</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>74608</v>
+        <v>70590</v>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
     </row>

</xml_diff>